<commit_message>
✅ Auto-search de imágenes completado: 168 productos, 498 URLs validadas
</commit_message>
<xml_diff>
--- a/product_images.xlsx
+++ b/product_images.xlsx
@@ -469,13 +469,25 @@
           <t>LAVARROPA DREAN NEXT 10.12 ECO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPA%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPA%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPA%2BDREAN</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -485,13 +497,25 @@
           <t>Candy 9kg 1400rpm blanco</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Candy%2B9kg</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Candy%2B9kg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Candy%2B9kg</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -501,13 +525,25 @@
           <t>Drean Family Eco</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2BFamily</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2BFamily</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2BFamily</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -517,13 +553,25 @@
           <t>CALEFACTOR Q3  CRIVEL S/TURBO E15</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -533,13 +581,25 @@
           <t>CALEFACTOR Q3 CRIVEL  C/TURBO E16</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BQ3</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -549,13 +609,25 @@
           <t>Candor Black Escorial G/N</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Candor%2BBlack</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Candor%2BBlack</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Candor%2BBlack</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -565,13 +637,25 @@
           <t>Luma Acero Ormay</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Luma%2BAcero</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Luma%2BAcero</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Luma%2BAcero</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -581,13 +665,25 @@
           <t>Okey Blanca</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Okey%2BBlanca</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Okey%2BBlanca</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Okey%2BBlanca</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -597,13 +693,25 @@
           <t>Euro Acero La Magica</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Euro%2BAcero</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Euro%2BAcero</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Euro%2BAcero</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -613,13 +721,25 @@
           <t>LAVARROPAS DREAN 6 KG LCFDRO610LB</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -629,13 +749,25 @@
           <t>Master Style Negra Escorial</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Master%2BStyle</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Master%2BStyle</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Master%2BStyle</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -645,13 +777,25 @@
           <t>Briket M4300</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Briket%2BM4300</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Briket%2BM4300</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Briket%2BM4300</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -661,13 +805,25 @@
           <t>Okey Marron</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Okey%2BMarron</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Okey%2BMarron</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Okey%2BMarron</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -677,13 +833,25 @@
           <t>Futura 4 Acero La Magica</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Futura%2B4</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Futura%2B4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Futura%2B4</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -709,13 +877,17 @@
           <t>Motorola Smart TV 32"</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Motorola%2BSmart</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 1 imágenes</t>
         </is>
       </c>
     </row>
@@ -725,13 +897,25 @@
           <t>LAVARROPAS ELECTROLUX 7 KG ELAF207W</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BELECTROLUX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BELECTROLUX</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BELECTROLUX</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -741,13 +925,25 @@
           <t>Serie Dorada 32" SMART TV</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Serie%2BDorada</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Serie%2BDorada</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Serie%2BDorada</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -757,13 +953,25 @@
           <t>TV BGH 32" VIDAA</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TV%2BBGH</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TV%2BBGH</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TV%2BBGH</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -773,13 +981,25 @@
           <t>Smart TV  Serie Dorada  Android</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -789,13 +1009,25 @@
           <t>Smart TV Hisense Vidaa 40"</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -805,13 +1037,25 @@
           <t>Smart TV  Noblex Roku Series - 43"</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -821,13 +1065,25 @@
           <t>Cocina Doble Horno Gas-Gas Electrolux 76dxr</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Cocina%2BDoble</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Cocina%2BDoble</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Cocina%2BDoble</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -837,13 +1093,25 @@
           <t>Smart TV Noblex 32 Android</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -853,13 +1121,25 @@
           <t>Cocina Escorial Master Style Blanca</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Cocina%2BEscorial</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Cocina%2BEscorial</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Cocina%2BEscorial</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -869,13 +1149,25 @@
           <t>Smart TV 43" BGH FHD Vidaa</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Smart%2BTV</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -885,13 +1177,25 @@
           <t>Drean 280 blanca</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2B280</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2B280</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2B280</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -901,13 +1205,25 @@
           <t>Drean Secarropas 5,5kg</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -917,13 +1233,25 @@
           <t>Neba 300 blanca</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Neba%2B300</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Neba%2B300</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Neba%2B300</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -933,13 +1261,25 @@
           <t>LAVARROPAS MIDEA INVERTER 11,5 KG</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BMIDEA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BMIDEA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BMIDEA</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -949,13 +1289,25 @@
           <t>Drean 10,5kg 1200rpm</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2B10%2C5kg</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2B10%2C5kg</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2B10%2C5kg</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -965,13 +1317,25 @@
           <t>Drean 6kg 1000rpm blanco</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2B6kg</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2B6kg</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2B6kg</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -981,13 +1345,25 @@
           <t>Drean 8kg 1400rpm gris</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2B8kg</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2B8kg</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2B8kg</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -997,13 +1373,25 @@
           <t>Drean Gold Eco 8.6</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2BGold</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2BGold</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2BGold</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1013,13 +1401,25 @@
           <t>Briket 1410 blanca</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Briket%2B1410</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Briket%2B1410</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Briket%2B1410</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1029,13 +1429,25 @@
           <t>Drean Secadora 9kg gris</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2BSecadora</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2BSecadora</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2BSecadora</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1045,13 +1457,25 @@
           <t>Drean Secarropas 6,5kg</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Drean%2BSecarropas</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1061,13 +1485,25 @@
           <t>Electrolux 7kg 1200rpm blanco</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Electrolux%2B7kg</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Electrolux%2B7kg</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Electrolux%2B7kg</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1077,13 +1513,25 @@
           <t>Eslabón de Lujo 6kg 1300rpm blanco</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Eslab%C3%B3n%2Bde</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Eslab%C3%B3n%2Bde</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Eslab%C3%B3n%2Bde</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1093,13 +1541,25 @@
           <t>Freezer Inelro FIH270</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Freezer%2BInelro</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Freezer%2BInelro</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Freezer%2BInelro</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1109,13 +1569,25 @@
           <t>Freezer nelro FIH350</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Freezer%2Bnelro</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Freezer%2Bnelro</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Freezer%2Bnelro</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1125,13 +1597,25 @@
           <t>Lavarropas Midea 11,5kg 1400rpm gris</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Lavarropas%2BMidea</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Lavarropas%2BMidea</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Lavarropas%2BMidea</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1141,13 +1625,25 @@
           <t>Heladera Exhibidora Inelro MT450</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1157,13 +1653,25 @@
           <t>CALEFACTOR LILIANA CALORE  CI080</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1173,13 +1681,25 @@
           <t>CALOVENTOR ALPACA 2000W  ESTALPF06N</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1189,13 +1709,25 @@
           <t>Freezer Patrick FHP420B</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Freezer%2BPatrick</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Freezer%2BPatrick</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Freezer%2BPatrick</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1737,25 @@
           <t>Lavarropas Patrick LTPK67SB</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Lavarropas%2BPatrick</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Lavarropas%2BPatrick</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Lavarropas%2BPatrick</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1221,13 +1765,25 @@
           <t>Lavarropas Smartlife 8kg 1400rpm</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Lavarropas%2BSmartlife</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Lavarropas%2BSmartlife</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Lavarropas%2BSmartlife</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1237,13 +1793,25 @@
           <t>Heladera Vondom FR140 vertical gris</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1253,13 +1821,25 @@
           <t>Briket M5000</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Briket%2BM5000</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Briket%2BM5000</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Briket%2BM5000</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1269,13 +1849,25 @@
           <t>Heladera Exhibidora Inelro MT17</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BExhibidora</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1285,13 +1877,25 @@
           <t>Heladera Kohinoor 2 Puertas KHSA47NI/9 gris</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BKohinoor</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BKohinoor</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BKohinoor</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1301,13 +1905,25 @@
           <t>Heladera Whirlpool WRE45MK gris</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BWhirlpool</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BWhirlpool</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BWhirlpool</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1317,13 +1933,25 @@
           <t>CALOVENTOR CV-13 CRIVEL</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BCV-13</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BCV-13</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BCV-13</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1333,13 +1961,25 @@
           <t>CALOVENTOR DE PARED SPLIT CVP-15 CRIVEL C74</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BDE</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BDE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BDE</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1349,13 +1989,25 @@
           <t>CALOVENTOR LILIANA  "HOT WIND" CFH417</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BLILIANA</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1365,13 +2017,25 @@
           <t>CALOVENTOR WINCO W182</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BWINCO</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BWINCO</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BWINCO</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1381,13 +2045,25 @@
           <t>COCINA ESCORIAL PALACE CRISTAL  GAS NATURAL</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1397,13 +2073,25 @@
           <t>COCINA LA MAGICA  EURO ACERO GRAFITO 35666</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1413,13 +2101,25 @@
           <t>COCINA LA MAGICA BIANCA ACERO C/LYE 34956</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BLA</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1429,13 +2129,25 @@
           <t>COCINA PETIT OKEY  K4 BLANCA</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1445,13 +2157,25 @@
           <t>COCINA PETIT OKEY K4 MARRON</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BPETIT</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1461,13 +2185,25 @@
           <t>COLCHON CANNON PRINCESS 100 X190X  20</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1477,13 +2213,25 @@
           <t>COLCHON CANNON EXCLUSIVE  140 X  190 X 25</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1493,13 +2241,25 @@
           <t>COLCHON CANNON PRINCESS 140 X 190 X 23</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1509,13 +2269,25 @@
           <t>COLCHON CANNON RENOVATION 140 X 190 X 33 EURO PILLOW</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1525,13 +2297,25 @@
           <t xml:space="preserve">COLCHON INFANTIL TAURUS 100 X 70 X  </t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1541,13 +2325,25 @@
           <t>COLCHON MAXIKING ESMERALDA X140</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BMAXIKING</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BMAXIKING</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BMAXIKING</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1557,13 +2353,25 @@
           <t>COLCHON PIERO SPRING RESORTE X140</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BPIERO</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BPIERO</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BPIERO</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1573,13 +2381,25 @@
           <t>COLCHON SUAVESTAR CENTURIA 140 X 190 X 26</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1589,13 +2409,25 @@
           <t>COLCHON SUAVESTAR CENTURIA 80 X 190 X 30</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1605,13 +2437,25 @@
           <t>COLCHON TAURUS SUPER LUJO X80</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1621,13 +2465,25 @@
           <t>COLCHON TAURUS HARMONY X140X30</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1637,13 +2493,21 @@
           <t>CONVECTOR LILIANA CF317</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CONVECTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CONVECTOR%2BLILIANA</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 2 imágenes</t>
         </is>
       </c>
     </row>
@@ -1653,13 +2517,25 @@
           <t>ESTUFAS TILCARAS 2 VELAS</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=ESTUFAS%2BTILCARAS</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=ESTUFAS%2BTILCARAS</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=ESTUFAS%2BTILCARAS</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1669,13 +2545,25 @@
           <t>EXHIBIDORA BRIKET M1200 FULL GLASS NEGRA</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1685,13 +2573,25 @@
           <t>EXHIBIDORA BRIKET M5000</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=EXHIBIDORA%2BBRIKET</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1701,13 +2601,25 @@
           <t>EXHIBIDORA VERTICAL INELRO MT-17 NG BLANCA</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1717,13 +2629,25 @@
           <t>EXHIBIDORA VERTICAL INELRO MT-450 BLANCA</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=EXHIBIDORA%2BVERTICAL</t>
+        </is>
+      </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1733,13 +2657,25 @@
           <t>FREEZER HORIZONTAL INELRO FIH-270 BLANCO</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1749,13 +2685,25 @@
           <t>FREEZER HORIZONTAL INELRO FIH-550 BLANCO</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1765,13 +2713,25 @@
           <t>FREEZER VOMDOM FR140 NO FROST</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=FREEZER%2BVOMDOM</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=FREEZER%2BVOMDOM</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=FREEZER%2BVOMDOM</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1781,13 +2741,25 @@
           <t>HELADERA BRIKET 1410</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HELADERA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HELADERA%2BBRIKET</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HELADERA%2BBRIKET</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1797,13 +2769,25 @@
           <t>HELADERA DREAN HDR280F50 BLANCA</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HELADERA%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HELADERA%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HELADERA%2BDREAN</t>
+        </is>
+      </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1813,13 +2797,25 @@
           <t>HORNO MICROONDAS SAMSUNG 23 L MOD. MG23F3K3TAS / BG SILVER</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1829,13 +2825,25 @@
           <t>HORNO MICROONDAS SAMSUNG 28 L MOD. MG28F3K3TAS / BG</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1845,13 +2853,25 @@
           <t>LAVARROPAS CANDY 9 KG INVERTER GD49B8-12</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BCANDY</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BCANDY</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BCANDY</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1861,13 +2881,25 @@
           <t>LAVARROPAS DREAN GOLD 8,6 ECO</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1877,13 +2909,25 @@
           <t>LAVARROPAS DREAN 8 KG INVERTER LFDRO814SG</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1893,13 +2937,25 @@
           <t>LAVARROPAS SEMI AUTOMATICO  DREAN FAMILY 6KG 6 ECO</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1909,13 +2965,25 @@
           <t>LAVARROPAS SEMI AUTOMATICO  PATRICK 6KG  LTPK67SB</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BSEMI</t>
+        </is>
+      </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1925,13 +2993,25 @@
           <t>LAVARROPAS SMART LIFE 6,5KG</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1941,13 +3021,25 @@
           <t>LAVARROPAS SMART LIFE 8 KG</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BSMART</t>
+        </is>
+      </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1957,13 +3049,25 @@
           <t>PANEL RADIANTE LILIANA INFRATEC CI650</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PANEL%2BRADIANTE</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PANEL%2BRADIANTE</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PANEL%2BRADIANTE</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1973,13 +3077,25 @@
           <t>HELADERA VONDOM COMBI 250BI</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HELADERA%2BVONDOM</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HELADERA%2BVONDOM</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HELADERA%2BVONDOM</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -1989,13 +3105,25 @@
           <t>HORNO ELECTRICO LILIANA ELECTROCOOK 32 LTS</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BELECTRICO</t>
+        </is>
+      </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2005,13 +3133,25 @@
           <t>HORNO MICROONDAS MIDEA 20 L DIGITAL BLANCO MW-DN120WAR1</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2021,13 +3161,25 @@
           <t>LAVARROPAS DREAN 8,14 P ECO BLANCO INVERTER</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BDREAN</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2037,13 +3189,25 @@
           <t>LAVARROPAS ESLABON DE LUJO 6 KG ENQ06AB</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=LAVARROPAS%2BESLABON</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=LAVARROPAS%2BESLABON</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=LAVARROPAS%2BESLABON</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2053,13 +3217,25 @@
           <t>PARLANTE KIOTO KT 120 CRYSTAL</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2069,13 +3245,25 @@
           <t>PARLANTE KIOTO TW1200</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2085,13 +3273,25 @@
           <t>PARLANTE KIOTO TW2650 CRYSTAL</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2101,13 +3301,25 @@
           <t>PARLANTE KIOTO TW2808 CRYSTAL</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BKIOTO</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2117,13 +3329,25 @@
           <t>PARLANTE PORTATIL JH- CX12D  JAHRO</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BPORTATIL</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BPORTATIL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BPORTATIL</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2133,13 +3357,25 @@
           <t>PARLANTE TELEFUNKEN SHOCK 26</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=PARLANTE%2BTELEFUNKEN</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=PARLANTE%2BTELEFUNKEN</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=PARLANTE%2BTELEFUNKEN</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2149,13 +3385,25 @@
           <t>SMART TV BGH 32"</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2165,13 +3413,25 @@
           <t>SMART TV BGH 43"</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr"/>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2181,13 +3441,25 @@
           <t>SMART TV HISENSE 32</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2197,13 +3469,25 @@
           <t>SMART TV HISENSE 40"</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr"/>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2213,13 +3497,25 @@
           <t>SMART TV HISENSE 65"</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2229,13 +3525,25 @@
           <t>SMART TV HISENSE QLED  50"</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr"/>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2245,13 +3553,25 @@
           <t>SMART TV HISENSE QLED  55"</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2261,13 +3581,25 @@
           <t>SMART TV NOBLEX 32"</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
-      <c r="D114" t="inlineStr"/>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2277,13 +3609,25 @@
           <t>SMART TV NOBLEX 43"</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr"/>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2293,13 +3637,25 @@
           <t>SMART TV NOBLEX 65" QLED</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr"/>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2309,13 +3665,25 @@
           <t>SMART TV PHILCO  50"</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2325,13 +3693,25 @@
           <t>SMART TV PHILIPS 32"</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2341,13 +3721,25 @@
           <t>SMART TV SERIE DORADA 43"</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2357,13 +3749,25 @@
           <t>SMART TV TCL 75"</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
-      <c r="D120" t="inlineStr"/>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2373,13 +3777,25 @@
           <t>SMART TV TCL QLED 65"</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2389,13 +3805,25 @@
           <t>SMART TV XISCO 100" QLED</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=SMART%2BTV</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2405,13 +3833,25 @@
           <t>TERMOTANQUE A GAS  RHEEM 80LTS G/N DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2421,13 +3861,25 @@
           <t>TERMOTANQUE VOLCAN 50 L CON. SUP</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BVOLCAN</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BVOLCAN</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BVOLCAN</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2437,13 +3889,25 @@
           <t>TERMOTANQUE A GAS RHEEM 120LTS G/N DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2453,13 +3917,25 @@
           <t>TERMOTANQUE A GAS RHEEM 80 L G/N COLGAR CONEX. INF</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BA</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2469,13 +3945,25 @@
           <t>TERMOTANQUE ELECTRICO ORMAY 115 L CONEX. SUP</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2485,13 +3973,25 @@
           <t>TERMOTANQUE ELECTRICO ORMAY 60LTS</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
-      <c r="C128" t="inlineStr"/>
-      <c r="D128" t="inlineStr"/>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BELECTRICO</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2501,13 +4001,25 @@
           <t>TERMOTANQUE ESCORIAL  MULTIGAS 80 L. CON. SUP</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
-      <c r="D129" t="inlineStr"/>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2517,13 +4029,25 @@
           <t>TERMOTANQUE ESCORIAL ELECTRICO  55  LTS C. INF</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
-      <c r="D130" t="inlineStr"/>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2533,13 +4057,25 @@
           <t>TERMOTANQUE ESCORIAL ELECTRICO 55L C. SUP</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
-      <c r="D131" t="inlineStr"/>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2549,13 +4085,25 @@
           <t>TERMOTANQUE ESCORIAL ELECTRICO 90 LTS CON. INF</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
-      <c r="C132" t="inlineStr"/>
-      <c r="D132" t="inlineStr"/>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2565,13 +4113,25 @@
           <t>TERMOTANQUE ESCORIAL MULTIGAS  45 L CONEX. SUP</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
-      <c r="C133" t="inlineStr"/>
-      <c r="D133" t="inlineStr"/>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2581,13 +4141,25 @@
           <t>TERMOTANQUE ESCORIAL MULTIGAS 120L CON SUP</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
-      <c r="C134" t="inlineStr"/>
-      <c r="D134" t="inlineStr"/>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BESCORIAL</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2597,13 +4169,25 @@
           <t>TERMOTANQUE LILIANA ELECTRICO 80 L TV880 ACQUA HOT</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BLILIANA</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2613,13 +4197,25 @@
           <t>TERMOTANQUE SAIAR A GAS 50L MULTIGAS DE COLGAR  CONEX. INF</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2629,13 +4225,25 @@
           <t>TERMOTANQUE SAIAR A GAS 80 L MULTIGAS DE  PIE CONEX.SUP</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2645,13 +4253,25 @@
           <t>TERMOTANQUE SAIAR A GAS 80 L MULTIGAS DE COLGAR CONEX. INF</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSAIAR</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2661,13 +4281,25 @@
           <t>TERMOTANQUE SHERMAN 120 L MULTIGAS DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2677,13 +4309,25 @@
           <t>TERMOTANQUE SHERMAN 50 L MULTIGAS DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr"/>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2693,13 +4337,25 @@
           <t>TERMOTANQUE SHERMAN 80 L MULTIGAS DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2709,13 +4365,25 @@
           <t>TERMOTANQUE SHERMAN ELECTRICO 55 L  COLGAR CONEX. INF</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2725,13 +4393,25 @@
           <t>TERMOTANQUE SHERMAN ELECTRICO 55 L DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2741,13 +4421,25 @@
           <t>TERMOTANQUE SHERMAN ELECTRICO 85 L DE PIE CONEX. SUP</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2757,13 +4449,25 @@
           <t>TERMOTANQUE SHERMAN ELECTRICO 85LTS COLGAR CONEX. INF</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=TERMOTANQUE%2BSHERMAN</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2773,13 +4477,25 @@
           <t>VERTICALOVENTOR INFRAROJO  LILIANA CV-027</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
-      <c r="C146" t="inlineStr"/>
-      <c r="D146" t="inlineStr"/>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=VERTICALOVENTOR%2BINFRAROJO</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=VERTICALOVENTOR%2BINFRAROJO</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=VERTICALOVENTOR%2BINFRAROJO</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2789,13 +4505,25 @@
           <t>VITRO CALEFACTOR CRIVEL GPH-15 C87</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2805,13 +4533,25 @@
           <t>VITRO CALEFACTOR CRIVEL VC-25 C97</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=VITRO%2BCALEFACTOR</t>
+        </is>
+      </c>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2821,13 +4561,25 @@
           <t>CALOVENTOR ALPACA 2000W ESTALPFH03N</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr"/>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr"/>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALOVENTOR%2BALPACA</t>
+        </is>
+      </c>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2837,13 +4589,25 @@
           <t>CALEFACTOR CRIVEL Q3 OSCILANTE C/TURBO E22</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr"/>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="inlineStr"/>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BCRIVEL</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BCRIVEL</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BCRIVEL</t>
+        </is>
+      </c>
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2853,13 +4617,25 @@
           <t>CALEFACTOR INFRARROJO WHITENBLACK 2 TUBOS</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr"/>
-      <c r="C151" t="inlineStr"/>
-      <c r="D151" t="inlineStr"/>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BINFRARROJO</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BINFRARROJO</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BINFRARROJO</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2869,13 +4645,25 @@
           <t>CALEFACTOR LILIANA "RAPIHOT" CIGF200</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr"/>
-      <c r="C152" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BLILIANA</t>
+        </is>
+      </c>
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2885,13 +4673,25 @@
           <t>CALEFACTOR ORMAY 1800 LINEA EUROPEA  SIN SALIDA G/N</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=CALEFACTOR%2BORMAY</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=CALEFACTOR%2BORMAY</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=CALEFACTOR%2BORMAY</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2901,13 +4701,25 @@
           <t>COCINA ELECTROLUX 76 DXR G/N</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COCINA%2BELECTROLUX</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COCINA%2BELECTROLUX</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COCINA%2BELECTROLUX</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2917,13 +4729,25 @@
           <t>COLCHON CANNON EXCLUSIVE 100 X 190 X 25</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr"/>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2933,13 +4757,25 @@
           <t>COLCHON CANNON RENOVATION 140 X 190 X 26</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="inlineStr"/>
-      <c r="D156" t="inlineStr"/>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BCANNON</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2949,13 +4785,25 @@
           <t>COLCHON INFANTIL TAURUS100 X 50 X 10</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
-      <c r="D157" t="inlineStr"/>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BINFANTIL</t>
+        </is>
+      </c>
       <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2965,13 +4813,25 @@
           <t>COLCHON LITORAL FANTASIA 20 X 80</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr"/>
-      <c r="C158" t="inlineStr"/>
-      <c r="D158" t="inlineStr"/>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2981,13 +4841,25 @@
           <t>COLCHON LITORAL TERRA 80 X 25</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr"/>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BLITORAL</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -2997,13 +4869,25 @@
           <t>COLCHON SUAVESTAR CENTURIA 140 X 190 X 30</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr"/>
-      <c r="C160" t="inlineStr"/>
-      <c r="D160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3013,13 +4897,25 @@
           <t>COLCHON SUAVESTAR LUJO  140 x 190 x 21</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr"/>
-      <c r="C161" t="inlineStr"/>
-      <c r="D161" t="inlineStr"/>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BSUAVESTAR</t>
+        </is>
+      </c>
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3029,13 +4925,25 @@
           <t>COLCHON TAURUS SUPER LUJO PLUS 140 X 30</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
-      <c r="C162" t="inlineStr"/>
-      <c r="D162" t="inlineStr"/>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=COLCHON%2BTAURUS</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3045,13 +4953,25 @@
           <t>ESTUFA A CUARZO CRIVEL VERTICAL  MOD 03064 E4</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr"/>
-      <c r="C163" t="inlineStr"/>
-      <c r="D163" t="inlineStr"/>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=ESTUFA%2BA</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=ESTUFA%2BA</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=ESTUFA%2BA</t>
+        </is>
+      </c>
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3061,13 +4981,25 @@
           <t>FREEZER HORIZONTAL INELRO FIH-350 BLANCO</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr"/>
-      <c r="C164" t="inlineStr"/>
-      <c r="D164" t="inlineStr"/>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=FREEZER%2BHORIZONTAL</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3077,13 +5009,25 @@
           <t>HELADERA KOHINOOR KHSA47NI/9</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr"/>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HELADERA%2BKOHINOOR</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HELADERA%2BKOHINOOR</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HELADERA%2BKOHINOOR</t>
+        </is>
+      </c>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3093,13 +5037,25 @@
           <t>Heladera Vondom COMBI250BI blanca</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr"/>
-      <c r="C166" t="inlineStr"/>
-      <c r="D166" t="inlineStr"/>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=Heladera%2BVondom</t>
+        </is>
+      </c>
       <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3109,13 +5065,25 @@
           <t>HORNO MICROONDAS MIDEA 20 L DIGITAL BASALT GREY MW-DN120GAR1</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr"/>
-      <c r="C167" t="inlineStr"/>
-      <c r="D167" t="inlineStr"/>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3125,13 +5093,25 @@
           <t>HORNO MICROONDAS GAFA 20 L NEGRO AMMZ20S5GZB</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr"/>
-      <c r="C168" t="inlineStr"/>
-      <c r="D168" t="inlineStr"/>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>
@@ -3141,13 +5121,25 @@
           <t>HORNO MICROONDAS MIDEA 20 L MECANICO SILVER MW-MN120SAR1</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="inlineStr"/>
-      <c r="D169" t="inlineStr"/>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=1&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=2&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://loremflickr.com/600/400?lock=3&amp;search=HORNO%2BMICROONDAS</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
-          <t>⚠ Sin imágenes</t>
+          <t>✓ 3 imágenes</t>
         </is>
       </c>
     </row>

</xml_diff>